<commit_message>
Update Task 5, 6, 7, 8
</commit_message>
<xml_diff>
--- a/Task_05/DucNVFX14814_CN1_Review_Checklist.xlsx
+++ b/Task_05/DucNVFX14814_CN1_Review_Checklist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Funix\4. CC4\5. LAB301x\LAB301x_01\Task_05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECB97A8E-7820-4D23-AA50-CF213A3EF4E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A7CDDBE-0CCF-4C28-AD1F-EDAD5B6FAF00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -108,10 +108,10 @@
     <t>CHECKLIST TỰ KIỂM TRA - TASK 5: CN1 QUẢN LÝ NGƯỜI DÙNG</t>
   </si>
   <si>
-    <t>Đã tạo các unit test và chạy cho các lớp DAO</t>
-  </si>
-  <si>
-    <t>Đã tạo các unit test và chạy cho các lớp DAO, đầy đủ các method được dùng trong hệ thống</t>
+    <t>Đã tạo các unit test và chạy cho các lớp DAO và BO</t>
+  </si>
+  <si>
+    <t>Đã tạo các unit test và chạy cho các lớp DAO và BO, đầy đủ các method được dùng trong hệ thống</t>
   </si>
 </sst>
 </file>
@@ -241,15 +241,15 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -530,25 +530,25 @@
     <col min="7" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:6" s="7" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-    </row>
-    <row r="2" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+    </row>
+    <row r="2" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -740,7 +740,7 @@
       <c r="C17" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="8">
         <f>COUNTA(E5:E15)</f>
         <v>11</v>
       </c>
@@ -749,7 +749,7 @@
       <c r="C18" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="8">
         <f>COUNTIF(E5:E15,"Đã thực hiện")</f>
         <v>11</v>
       </c>
@@ -758,7 +758,7 @@
       <c r="C19" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="8">
         <f>COUNTIF(E5:E15,"Chưa thực hiện")</f>
         <v>0</v>
       </c>

</xml_diff>